<commit_message>
changed plot presence for misidentified species
</commit_message>
<xml_diff>
--- a/tocheck/plotsbci_not_garwood_2026-04-30.xlsx
+++ b/tocheck/plotsbci_not_garwood_2026-04-30.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BL15"/>
+  <dimension ref="A1:BL16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -412,17 +412,17 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>bci25ha</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>AVA</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Zetek</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>bci25ha</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>AVA</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="BK2">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BL2" t="inlineStr">
         <is>
@@ -2878,13 +2878,13 @@
         <v>4</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11">
         <v>0</v>
@@ -3088,7 +3088,7 @@
         </is>
       </c>
       <c r="BK11">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="BL11" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="BK12">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="BL12" t="inlineStr">
         <is>
@@ -3572,7 +3572,7 @@
         </is>
       </c>
       <c r="BK13">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="BL13" t="inlineStr">
         <is>
@@ -3619,13 +3619,13 @@
         <v>0</v>
       </c>
       <c r="L14">
+        <v>21</v>
+      </c>
+      <c r="M14">
+        <v>44</v>
+      </c>
+      <c r="N14">
         <v>37</v>
-      </c>
-      <c r="M14">
-        <v>21</v>
-      </c>
-      <c r="N14">
-        <v>44</v>
       </c>
       <c r="O14">
         <v>31</v>
@@ -3824,7 +3824,7 @@
         </is>
       </c>
       <c r="BK14">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="BL14" t="inlineStr">
         <is>
@@ -3835,240 +3835,487 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>unonpa</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>1</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15" t="b">
+        <v>1</v>
+      </c>
+      <c r="T15" t="b">
+        <v>0</v>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Zetek</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Magnoliales</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Annonaceae</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Unonopsis</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>panamensis</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>R.E. Fr.</t>
+        </is>
+      </c>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>R. Pérez 2303 (PMA, SCZ)</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Freestanding</t>
+        </is>
+      </c>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>unonpa</t>
+        </is>
+      </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>species</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>R.E.Fr.</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>2447472</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>259517-2</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>2447472</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>259517-2</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>259517-2</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>R.E.Fr.</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>Annonaceae</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>Unonopsis</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>panamensis</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>Species</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BG15" t="inlineStr">
+        <is>
+          <t>UNO2</t>
+        </is>
+      </c>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+      <c r="BI15" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>Plots_census</t>
+        </is>
+      </c>
+      <c r="BK15">
+        <v>359</v>
+      </c>
+      <c r="BL15" t="inlineStr">
+        <is>
+          <t>Unonopsis panamensis</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>viroel</t>
         </is>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+      <c r="F16">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
         <v>3</v>
       </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>0</v>
-      </c>
-      <c r="R15">
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
         <v>34</v>
       </c>
-      <c r="S15" t="b">
-        <v>0</v>
-      </c>
-      <c r="T15" t="b">
-        <v>1</v>
-      </c>
-      <c r="U15" t="inlineStr">
+      <c r="S16" t="b">
+        <v>0</v>
+      </c>
+      <c r="T16" t="b">
+        <v>1</v>
+      </c>
+      <c r="U16" t="inlineStr">
         <is>
           <t>gigante1, gigante_plot</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>Magnoliales</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>Myristicaceae</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>Virola</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>elongata</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr">
+      <c r="AA16" t="inlineStr">
         <is>
           <t>(Benth.) Warb.</t>
         </is>
       </c>
-      <c r="AD15" t="inlineStr">
+      <c r="AD16" t="inlineStr">
         <is>
           <t>Freestanding</t>
         </is>
       </c>
-      <c r="AE15" t="inlineStr">
+      <c r="AE16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="AF15" t="inlineStr">
+      <c r="AF16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="AH15" t="inlineStr">
+      <c r="AH16" t="inlineStr">
         <is>
           <t>viroel</t>
         </is>
       </c>
-      <c r="AI15" t="inlineStr">
+      <c r="AI16" t="inlineStr">
         <is>
           <t>species</t>
         </is>
       </c>
-      <c r="AJ15" t="inlineStr">
+      <c r="AJ16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="AK15" t="inlineStr">
+      <c r="AK16" t="inlineStr">
         <is>
           <t>(Benth.) Warb.</t>
         </is>
       </c>
-      <c r="AL15" t="inlineStr">
+      <c r="AL16" t="inlineStr">
         <is>
           <t>Species</t>
         </is>
       </c>
-      <c r="AM15" t="inlineStr">
+      <c r="AM16" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="AN15" t="inlineStr">
+      <c r="AN16" t="inlineStr">
         <is>
           <t>2452056</t>
         </is>
       </c>
-      <c r="AO15" t="inlineStr">
+      <c r="AO16" t="inlineStr">
         <is>
           <t>267153-2</t>
         </is>
       </c>
-      <c r="AP15" t="inlineStr">
+      <c r="AP16" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AQ15" t="inlineStr">
+      <c r="AQ16" t="inlineStr">
         <is>
           <t>2452056</t>
         </is>
       </c>
-      <c r="AR15" t="inlineStr">
+      <c r="AR16" t="inlineStr">
         <is>
           <t>267153-2</t>
         </is>
       </c>
-      <c r="AS15" t="inlineStr">
+      <c r="AS16" t="inlineStr">
         <is>
           <t>267153-2</t>
         </is>
       </c>
-      <c r="AT15" t="inlineStr">
+      <c r="AT16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="AU15" t="inlineStr">
+      <c r="AU16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="AV15" t="inlineStr">
+      <c r="AV16" t="inlineStr">
         <is>
           <t>(Benth.) Warb.</t>
         </is>
       </c>
-      <c r="AW15" t="inlineStr">
+      <c r="AW16" t="inlineStr">
         <is>
           <t>Myristicaceae</t>
         </is>
       </c>
-      <c r="AX15" t="inlineStr">
+      <c r="AX16" t="inlineStr">
         <is>
           <t>Virola</t>
         </is>
       </c>
-      <c r="AY15" t="inlineStr">
+      <c r="AY16" t="inlineStr">
         <is>
           <t>elongata</t>
         </is>
       </c>
-      <c r="BB15" t="inlineStr">
+      <c r="BB16" t="inlineStr">
         <is>
           <t>Species</t>
         </is>
       </c>
-      <c r="BC15" t="inlineStr">
+      <c r="BC16" t="inlineStr">
         <is>
           <t>tree</t>
         </is>
       </c>
-      <c r="BD15" t="inlineStr">
+      <c r="BD16" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="BF15" t="inlineStr">
+      <c r="BF16" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="BG15" t="inlineStr">
+      <c r="BG16" t="inlineStr">
         <is>
           <t>VIRE</t>
         </is>
       </c>
-      <c r="BH15" t="inlineStr">
+      <c r="BH16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>
       </c>
-      <c r="BI15" t="b">
-        <v>1</v>
-      </c>
-      <c r="BJ15" t="inlineStr">
+      <c r="BI16" t="b">
+        <v>1</v>
+      </c>
+      <c r="BJ16" t="inlineStr">
         <is>
           <t>Plots_census</t>
         </is>
       </c>
-      <c r="BK15">
-        <v>365</v>
-      </c>
-      <c r="BL15" t="inlineStr">
+      <c r="BK16">
+        <v>364</v>
+      </c>
+      <c r="BL16" t="inlineStr">
         <is>
           <t>Virola elongata</t>
         </is>

</xml_diff>